<commit_message>
finales eis upload and extra upload check
</commit_message>
<xml_diff>
--- a/experiment_info_fc_uploader_schiedam.xlsx
+++ b/experiment_info_fc_uploader_schiedam.xlsx
@@ -1,31 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://battolyser-my.sharepoint.com/personal/c_hofman_alquion_com/Documents/Documenten/GitHub/clickhouse-uploader/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="11_F25DC773A252ABDACC1048D4C1D873BE5ADE58E9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C89CE975-3011-4694-AE6C-FBB9A47FB5DD}"/>
+  <xr:revisionPtr revIDLastSave="41" documentId="11_F25DC773A252ABDACC1048D4C1D873BE5ADE58E9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7BAC5C5-F125-4EDA-8FAD-09840A897A01}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="10">
   <si>
     <t>experiment_id</t>
   </si>
@@ -48,7 +59,13 @@
     <t>mmo_end_2</t>
   </si>
   <si>
-    <t>A20_C20</t>
+    <t>A6_C9</t>
+  </si>
+  <si>
+    <t>A6_C7</t>
+  </si>
+  <si>
+    <t>A5_C7</t>
   </si>
 </sst>
 </file>
@@ -366,19 +383,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -392,18 +409,18 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" t="s">
         <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
       </c>
       <c r="G1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>7</v>
@@ -412,39 +429,407 @@
         <v>1</v>
       </c>
       <c r="D2">
-        <v>-0.98699999999999999</v>
+        <v>-0.94299999999999995</v>
       </c>
       <c r="E2">
-        <v>-0.95399999999999996</v>
+        <v>-0.93500000000000005</v>
       </c>
       <c r="F2">
-        <v>-0.98699999999999999</v>
+        <v>-0.93700000000000006</v>
       </c>
       <c r="G2">
-        <v>-0.95399999999999996</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+        <v>-0.93700000000000006</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3">
-        <v>-0.98699999999999999</v>
+        <v>-0.93799999999999994</v>
       </c>
       <c r="E3">
-        <v>-0.95399999999999996</v>
+        <v>-0.94199999999999995</v>
       </c>
       <c r="F3">
-        <v>-0.98699999999999999</v>
+        <v>-0.93200000000000005</v>
       </c>
       <c r="G3">
-        <v>-0.95399999999999996</v>
+        <v>-0.93899999999999995</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4">
+        <v>-0.93600000000000005</v>
+      </c>
+      <c r="E4">
+        <v>-0.93400000000000005</v>
+      </c>
+      <c r="F4">
+        <v>-0.93300000000000005</v>
+      </c>
+      <c r="G4">
+        <v>-0.93899999999999995</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <v>4</v>
+      </c>
+      <c r="D5">
+        <v>-0.94799999999999995</v>
+      </c>
+      <c r="E5">
+        <v>-0.94399999999999995</v>
+      </c>
+      <c r="F5">
+        <v>-0.93899999999999995</v>
+      </c>
+      <c r="G5">
+        <v>-0.93400000000000005</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>-0.94299999999999995</v>
+      </c>
+      <c r="E6">
+        <v>-0.93300000000000005</v>
+      </c>
+      <c r="F6">
+        <v>-0.94299999999999995</v>
+      </c>
+      <c r="G6">
+        <v>-0.93300000000000005</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>2</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7">
+        <v>-0.93799999999999994</v>
+      </c>
+      <c r="E7">
+        <v>-0.92600000000000005</v>
+      </c>
+      <c r="F7">
+        <v>-0.93799999999999994</v>
+      </c>
+      <c r="G7">
+        <v>-0.92600000000000005</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>2</v>
+      </c>
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8">
+        <v>3</v>
+      </c>
+      <c r="D8">
+        <v>-0.93600000000000005</v>
+      </c>
+      <c r="E8">
+        <v>-0.93600000000000005</v>
+      </c>
+      <c r="F8">
+        <v>-0.93600000000000005</v>
+      </c>
+      <c r="G8">
+        <v>-0.93600000000000005</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>-0.93899999999999995</v>
+      </c>
+      <c r="E9">
+        <v>-0.93899999999999995</v>
+      </c>
+      <c r="F9">
+        <v>-0.93900000000000006</v>
+      </c>
+      <c r="G9">
+        <v>-0.94300000000000006</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10">
+        <v>2</v>
+      </c>
+      <c r="D10">
+        <v>-0.93700000000000006</v>
+      </c>
+      <c r="E10">
+        <v>-0.94299999999999995</v>
+      </c>
+      <c r="F10">
+        <v>-0.93500000000000005</v>
+      </c>
+      <c r="G10">
+        <v>-0.93500000000000005</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11">
+        <v>3</v>
+      </c>
+      <c r="D11">
+        <v>-0.93600000000000005</v>
+      </c>
+      <c r="E11">
+        <v>-0.93400000000000005</v>
+      </c>
+      <c r="F11">
+        <v>-0.93300000000000005</v>
+      </c>
+      <c r="G11">
+        <v>-0.92700000000000005</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12">
+        <v>-0.92800000000000005</v>
+      </c>
+      <c r="E12">
+        <v>-0.92900000000000005</v>
+      </c>
+      <c r="F12">
+        <v>-0.92500000000000004</v>
+      </c>
+      <c r="G12">
+        <v>-0.92</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>4</v>
+      </c>
+      <c r="B13" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13">
+        <v>2</v>
+      </c>
+      <c r="D13">
+        <v>-0.93500000000000005</v>
+      </c>
+      <c r="E13">
+        <v>-0.93500000000000005</v>
+      </c>
+      <c r="F13">
+        <v>-0.92800000000000005</v>
+      </c>
+      <c r="G13">
+        <v>-0.92100000000000004</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>4</v>
+      </c>
+      <c r="B14" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14">
+        <v>3</v>
+      </c>
+      <c r="D14">
+        <v>-0.93400000000000005</v>
+      </c>
+      <c r="E14">
+        <v>-0.93300000000000005</v>
+      </c>
+      <c r="F14">
+        <v>-0.93200000000000005</v>
+      </c>
+      <c r="G14">
+        <v>-0.93200000000000005</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>4</v>
+      </c>
+      <c r="B15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15">
+        <v>4</v>
+      </c>
+      <c r="D15">
+        <v>-0.92400000000000004</v>
+      </c>
+      <c r="E15">
+        <v>-0.93200000000000005</v>
+      </c>
+      <c r="F15">
+        <v>-0.93700000000000006</v>
+      </c>
+      <c r="G15">
+        <v>-0.92500000000000004</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>5</v>
+      </c>
+      <c r="B16" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16">
+        <v>-0.93</v>
+      </c>
+      <c r="E16">
+        <v>-0.92800000000000005</v>
+      </c>
+      <c r="F16">
+        <v>-0.92800000000000005</v>
+      </c>
+      <c r="G16">
+        <v>-0.98399999999999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>5</v>
+      </c>
+      <c r="B17" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17">
+        <v>2</v>
+      </c>
+      <c r="D17">
+        <v>-0.92900000000000005</v>
+      </c>
+      <c r="E17">
+        <v>-0.91</v>
+      </c>
+      <c r="F17">
+        <v>-0.92</v>
+      </c>
+      <c r="G17">
+        <v>-0.91800000000000004</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>5</v>
+      </c>
+      <c r="B18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18">
+        <v>3</v>
+      </c>
+      <c r="D18">
+        <v>-0.92800000000000005</v>
+      </c>
+      <c r="E18">
+        <v>-0.91200000000000003</v>
+      </c>
+      <c r="F18">
+        <v>-0.96799999999999997</v>
+      </c>
+      <c r="G18">
+        <v>-0.93799999999999994</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>5</v>
+      </c>
+      <c r="B19" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19">
+        <v>4</v>
+      </c>
+      <c r="D19">
+        <v>-0.92200000000000004</v>
+      </c>
+      <c r="E19">
+        <v>-0.93100000000000005</v>
+      </c>
+      <c r="F19">
+        <v>-0.98399999999999999</v>
+      </c>
+      <c r="G19">
+        <v>-0.93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>